<commit_message>
Final Update: Complete integration of Mechanical Status sheet in XLSX and JSON, restored Survey data, and updated production build
</commit_message>
<xml_diff>
--- a/app_unified/dist/PUMPS (1).xlsx
+++ b/app_unified/dist/PUMPS (1).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\OneDrive\Desktop\ESP DESING ESTUDIO\app_unified\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE71E1C4-371A-4A3E-948A-7EB0E44AD9FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6E36F49-F0FA-450F-9DEB-2D8748DE0FCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{FC341EB1-65C7-47F8-9E2D-590F22EBE9EA}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{FC341EB1-65C7-47F8-9E2D-590F22EBE9EA}"/>
   </bookViews>
   <sheets>
     <sheet name="PUMP" sheetId="1" r:id="rId1"/>
@@ -312,7 +312,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1456" uniqueCount="490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1521" uniqueCount="535">
   <si>
     <t>Required Pump data</t>
   </si>
@@ -1737,9 +1737,6 @@
     <t>-1.86E-19</t>
   </si>
   <si>
-    <t>SLB</t>
-  </si>
-  <si>
     <t>S4000N</t>
   </si>
   <si>
@@ -1834,6 +1831,144 @@
   </si>
   <si>
     <t>0.875</t>
+  </si>
+  <si>
+    <t>Schlumberger</t>
+  </si>
+  <si>
+    <t>DN 1050</t>
+  </si>
+  <si>
+    <t>71.2</t>
+  </si>
+  <si>
+    <t>55.42</t>
+  </si>
+  <si>
+    <t>-0.01152</t>
+  </si>
+  <si>
+    <t>0.125</t>
+  </si>
+  <si>
+    <t>0.0001845</t>
+  </si>
+  <si>
+    <t>5.12e-15</t>
+  </si>
+  <si>
+    <t>4.00</t>
+  </si>
+  <si>
+    <t>0.688</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>1.0</t>
+  </si>
+  <si>
+    <t>DN 1400</t>
+  </si>
+  <si>
+    <t>72.5</t>
+  </si>
+  <si>
+    <t>48.65</t>
+  </si>
+  <si>
+    <t>-0.008542</t>
+  </si>
+  <si>
+    <t>4.85e-09</t>
+  </si>
+  <si>
+    <t>-8.24e-13</t>
+  </si>
+  <si>
+    <t>0.155</t>
+  </si>
+  <si>
+    <t>0.0002145</t>
+  </si>
+  <si>
+    <t>9.85e-08</t>
+  </si>
+  <si>
+    <t>-3.54e-11</t>
+  </si>
+  <si>
+    <t>73.8</t>
+  </si>
+  <si>
+    <t>42.15</t>
+  </si>
+  <si>
+    <t>-0.006425</t>
+  </si>
+  <si>
+    <t>-9.84e-06</t>
+  </si>
+  <si>
+    <t>3.12e-09</t>
+  </si>
+  <si>
+    <t>-5.45e-13</t>
+  </si>
+  <si>
+    <t>0.185</t>
+  </si>
+  <si>
+    <t>0.000245</t>
+  </si>
+  <si>
+    <t>8.12e-08</t>
+  </si>
+  <si>
+    <t>-2.85e-11</t>
+  </si>
+  <si>
+    <t>3.12e-15</t>
+  </si>
+  <si>
+    <t>DN 1750</t>
+  </si>
+  <si>
+    <t>DN 1800</t>
+  </si>
+  <si>
+    <t>74.2</t>
+  </si>
+  <si>
+    <t>41.5</t>
+  </si>
+  <si>
+    <t>-0.00585</t>
+  </si>
+  <si>
+    <t>-9.12e-06</t>
+  </si>
+  <si>
+    <t>2.85e-09</t>
+  </si>
+  <si>
+    <t>-4.95e-13</t>
+  </si>
+  <si>
+    <t>0.198</t>
+  </si>
+  <si>
+    <t>0.000258</t>
+  </si>
+  <si>
+    <t>7.45e-08</t>
+  </si>
+  <si>
+    <t>-2.42e-11</t>
+  </si>
+  <si>
+    <t>2.85e-15</t>
   </si>
 </sst>
 </file>
@@ -2802,7 +2937,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{053E6D0B-9E01-4484-8758-0E93695A87D4}">
-  <dimension ref="A1:AJ1105"/>
+  <dimension ref="A1:AJ1104"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="19.6640625" customWidth="1"/>
@@ -17876,14 +18011,14 @@
       </c>
     </row>
     <row r="153" spans="1:36" s="44" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A153" s="14" t="s">
-        <v>457</v>
+      <c r="A153" s="68" t="s">
+        <v>489</v>
       </c>
       <c r="B153" s="93">
         <v>538</v>
       </c>
       <c r="C153" s="93" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="D153" s="93">
         <v>1000</v>
@@ -17895,10 +18030,10 @@
         <v>6000</v>
       </c>
       <c r="G153" s="93" t="s">
+        <v>458</v>
+      </c>
+      <c r="H153" s="93" t="s">
         <v>459</v>
-      </c>
-      <c r="H153" s="93" t="s">
-        <v>460</v>
       </c>
       <c r="I153" s="93">
         <v>7500</v>
@@ -17907,43 +18042,43 @@
         <v>60</v>
       </c>
       <c r="K153" s="78" t="s">
+        <v>460</v>
+      </c>
+      <c r="L153" s="78" t="s">
         <v>461</v>
       </c>
-      <c r="L153" s="78" t="s">
+      <c r="M153" s="78" t="s">
         <v>462</v>
       </c>
-      <c r="M153" s="78" t="s">
+      <c r="N153" s="78" t="s">
         <v>463</v>
       </c>
-      <c r="N153" s="78" t="s">
+      <c r="O153" s="78" t="s">
         <v>464</v>
       </c>
-      <c r="O153" s="78" t="s">
+      <c r="P153" s="78" t="s">
         <v>465</v>
       </c>
-      <c r="P153" s="78" t="s">
+      <c r="Q153" s="78" t="s">
         <v>466</v>
       </c>
-      <c r="Q153" s="78" t="s">
+      <c r="R153" s="78" t="s">
         <v>467</v>
       </c>
-      <c r="R153" s="78" t="s">
+      <c r="S153" s="78" t="s">
         <v>468</v>
       </c>
-      <c r="S153" s="78" t="s">
+      <c r="T153" s="78" t="s">
         <v>469</v>
       </c>
-      <c r="T153" s="78" t="s">
+      <c r="U153" s="78" t="s">
         <v>470</v>
       </c>
-      <c r="U153" s="78" t="s">
+      <c r="V153" s="78" t="s">
         <v>471</v>
       </c>
-      <c r="V153" s="78" t="s">
+      <c r="W153" s="80" t="s">
         <v>472</v>
-      </c>
-      <c r="W153" s="80" t="s">
-        <v>473</v>
       </c>
       <c r="X153" s="100" t="s">
         <v>440</v>
@@ -17981,7 +18116,7 @@
         <v>538</v>
       </c>
       <c r="C154" s="93" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="D154" s="93">
         <v>200</v>
@@ -17993,10 +18128,10 @@
         <v>2250</v>
       </c>
       <c r="G154" s="93" t="s">
+        <v>474</v>
+      </c>
+      <c r="H154" s="93" t="s">
         <v>475</v>
-      </c>
-      <c r="H154" s="93" t="s">
-        <v>476</v>
       </c>
       <c r="I154" s="93">
         <v>3000</v>
@@ -18005,43 +18140,43 @@
         <v>60</v>
       </c>
       <c r="K154" s="78" t="s">
+        <v>476</v>
+      </c>
+      <c r="L154" s="78" t="s">
         <v>477</v>
       </c>
-      <c r="L154" s="78" t="s">
+      <c r="M154" s="78" t="s">
         <v>478</v>
       </c>
-      <c r="M154" s="78" t="s">
+      <c r="N154" s="78" t="s">
         <v>479</v>
       </c>
-      <c r="N154" s="78" t="s">
+      <c r="O154" s="78" t="s">
         <v>480</v>
       </c>
-      <c r="O154" s="78" t="s">
+      <c r="P154" s="78" t="s">
         <v>481</v>
       </c>
-      <c r="P154" s="78" t="s">
+      <c r="Q154" s="78" t="s">
         <v>482</v>
       </c>
-      <c r="Q154" s="78" t="s">
+      <c r="R154" s="78" t="s">
         <v>483</v>
       </c>
-      <c r="R154" s="78" t="s">
+      <c r="S154" s="78" t="s">
         <v>484</v>
       </c>
-      <c r="S154" s="78" t="s">
+      <c r="T154" s="78" t="s">
         <v>485</v>
       </c>
-      <c r="T154" s="78" t="s">
+      <c r="U154" s="78" t="s">
         <v>486</v>
       </c>
-      <c r="U154" s="78" t="s">
+      <c r="V154" s="78" t="s">
         <v>487</v>
       </c>
-      <c r="V154" s="78" t="s">
-        <v>488</v>
-      </c>
       <c r="W154" s="80" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="X154" s="100">
         <v>5627</v>
@@ -18050,7 +18185,7 @@
         <v>440</v>
       </c>
       <c r="Z154" s="82" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="AA154" s="100" t="s">
         <v>440</v>
@@ -18072,140 +18207,420 @@
       </c>
     </row>
     <row r="155" spans="1:36" s="44" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A155" s="68"/>
-      <c r="B155" s="93"/>
-      <c r="C155" s="93"/>
-      <c r="D155" s="93"/>
-      <c r="E155" s="93"/>
-      <c r="F155" s="93"/>
-      <c r="G155" s="93"/>
-      <c r="H155" s="93"/>
-      <c r="I155" s="93"/>
-      <c r="J155" s="72"/>
-      <c r="K155" s="78"/>
-      <c r="L155" s="78"/>
-      <c r="M155" s="78"/>
-      <c r="N155" s="78"/>
-      <c r="O155" s="78"/>
-      <c r="P155" s="78"/>
-      <c r="Q155" s="78"/>
-      <c r="R155" s="78"/>
-      <c r="S155" s="78"/>
-      <c r="T155" s="78"/>
-      <c r="U155" s="78"/>
-      <c r="V155" s="78"/>
-      <c r="W155" s="80"/>
-      <c r="X155" s="100"/>
-      <c r="Y155" s="100"/>
-      <c r="Z155" s="82"/>
-      <c r="AA155" s="100"/>
-      <c r="AB155" s="100"/>
-      <c r="AC155" s="101"/>
-      <c r="AD155" s="101"/>
-      <c r="AE155" s="101"/>
-      <c r="AF155" s="98"/>
+      <c r="A155" s="68" t="s">
+        <v>489</v>
+      </c>
+      <c r="B155" s="93">
+        <v>400</v>
+      </c>
+      <c r="C155" s="93" t="s">
+        <v>490</v>
+      </c>
+      <c r="D155" s="93">
+        <v>300</v>
+      </c>
+      <c r="E155" s="93">
+        <v>1050</v>
+      </c>
+      <c r="F155" s="93">
+        <v>1650</v>
+      </c>
+      <c r="G155" s="93" t="s">
+        <v>491</v>
+      </c>
+      <c r="H155" s="93" t="s">
+        <v>492</v>
+      </c>
+      <c r="I155" s="93">
+        <v>1800</v>
+      </c>
+      <c r="J155" s="72" t="s">
+        <v>492</v>
+      </c>
+      <c r="K155" s="78" t="s">
+        <v>493</v>
+      </c>
+      <c r="L155" s="78">
+        <v>-1.54E-2</v>
+      </c>
+      <c r="M155" s="78">
+        <v>6.2099999999999998E-6</v>
+      </c>
+      <c r="N155" s="78">
+        <v>-1.03E-9</v>
+      </c>
+      <c r="O155" s="78">
+        <v>0</v>
+      </c>
+      <c r="P155" s="78" t="s">
+        <v>494</v>
+      </c>
+      <c r="Q155" s="78" t="s">
+        <v>495</v>
+      </c>
+      <c r="R155" s="78">
+        <v>1.12E-4</v>
+      </c>
+      <c r="S155" s="78">
+        <v>-4.1299999999999999E-8</v>
+      </c>
+      <c r="T155" s="78" t="s">
+        <v>496</v>
+      </c>
+      <c r="U155" s="78">
+        <v>0</v>
+      </c>
+      <c r="V155" s="78" t="s">
+        <v>497</v>
+      </c>
+      <c r="W155" s="80">
+        <v>5000</v>
+      </c>
+      <c r="X155" s="100">
+        <v>6000</v>
+      </c>
+      <c r="Y155" s="100" t="s">
+        <v>498</v>
+      </c>
+      <c r="Z155" s="82">
+        <v>154</v>
+      </c>
+      <c r="AA155" s="100">
+        <v>240</v>
+      </c>
+      <c r="AB155" s="100">
+        <v>1</v>
+      </c>
+      <c r="AC155" s="101">
+        <v>400</v>
+      </c>
+      <c r="AD155" s="101">
+        <v>1</v>
+      </c>
+      <c r="AE155" s="101">
+        <v>105</v>
+      </c>
+      <c r="AF155" s="98" t="s">
+        <v>499</v>
+      </c>
+      <c r="AG155" s="44">
+        <v>1050</v>
+      </c>
+      <c r="AH155" s="44" t="s">
+        <v>500</v>
+      </c>
     </row>
     <row r="156" spans="1:36" s="44" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A156" s="68"/>
-      <c r="B156" s="93"/>
-      <c r="C156" s="93"/>
-      <c r="D156" s="93"/>
-      <c r="E156" s="93"/>
-      <c r="F156" s="93"/>
-      <c r="G156" s="93"/>
-      <c r="H156" s="93"/>
-      <c r="I156" s="93"/>
-      <c r="J156" s="72"/>
-      <c r="K156" s="78"/>
-      <c r="L156" s="78"/>
-      <c r="M156" s="78"/>
-      <c r="N156" s="78"/>
-      <c r="O156" s="78"/>
-      <c r="P156" s="78"/>
-      <c r="Q156" s="78"/>
-      <c r="R156" s="78"/>
-      <c r="S156" s="78"/>
-      <c r="T156" s="78"/>
-      <c r="U156" s="78"/>
-      <c r="V156" s="78"/>
-      <c r="W156" s="80"/>
-      <c r="X156" s="100"/>
-      <c r="Y156" s="100"/>
-      <c r="Z156" s="82"/>
-      <c r="AA156" s="100"/>
-      <c r="AB156" s="100"/>
-      <c r="AC156" s="101"/>
-      <c r="AD156" s="101"/>
-      <c r="AE156" s="101"/>
-      <c r="AF156" s="98"/>
+      <c r="A156" s="68" t="s">
+        <v>489</v>
+      </c>
+      <c r="B156" s="93">
+        <v>400</v>
+      </c>
+      <c r="C156" s="93" t="s">
+        <v>501</v>
+      </c>
+      <c r="D156" s="93">
+        <v>400</v>
+      </c>
+      <c r="E156" s="93">
+        <v>1400</v>
+      </c>
+      <c r="F156" s="93">
+        <v>2200</v>
+      </c>
+      <c r="G156" s="93" t="s">
+        <v>502</v>
+      </c>
+      <c r="H156" s="93" t="s">
+        <v>503</v>
+      </c>
+      <c r="I156" s="93">
+        <v>2500</v>
+      </c>
+      <c r="J156" s="72" t="s">
+        <v>503</v>
+      </c>
+      <c r="K156" s="78" t="s">
+        <v>504</v>
+      </c>
+      <c r="L156" s="78">
+        <v>-1.1299999999999999E-2</v>
+      </c>
+      <c r="M156" s="78" t="s">
+        <v>505</v>
+      </c>
+      <c r="N156" s="78" t="s">
+        <v>506</v>
+      </c>
+      <c r="O156" s="78">
+        <v>0</v>
+      </c>
+      <c r="P156" s="78" t="s">
+        <v>507</v>
+      </c>
+      <c r="Q156" s="78" t="s">
+        <v>508</v>
+      </c>
+      <c r="R156" s="78" t="s">
+        <v>509</v>
+      </c>
+      <c r="S156" s="78" t="s">
+        <v>510</v>
+      </c>
+      <c r="T156" s="78">
+        <v>4.2200000000000002E-12</v>
+      </c>
+      <c r="U156" s="78">
+        <v>0</v>
+      </c>
+      <c r="V156" s="78" t="s">
+        <v>497</v>
+      </c>
+      <c r="W156" s="80">
+        <v>5000</v>
+      </c>
+      <c r="X156" s="100">
+        <v>6000</v>
+      </c>
+      <c r="Y156" s="100" t="s">
+        <v>498</v>
+      </c>
+      <c r="Z156" s="82">
+        <v>154</v>
+      </c>
+      <c r="AA156" s="100">
+        <v>240</v>
+      </c>
+      <c r="AB156" s="100">
+        <v>1</v>
+      </c>
+      <c r="AC156" s="101">
+        <v>400</v>
+      </c>
+      <c r="AD156" s="101">
+        <v>1</v>
+      </c>
+      <c r="AE156" s="101">
+        <v>163</v>
+      </c>
+      <c r="AF156" s="98" t="s">
+        <v>499</v>
+      </c>
+      <c r="AG156" s="44">
+        <v>1400</v>
+      </c>
+      <c r="AH156" s="44" t="s">
+        <v>500</v>
+      </c>
     </row>
     <row r="157" spans="1:36" s="44" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A157" s="68"/>
-      <c r="B157" s="93"/>
-      <c r="C157" s="93"/>
-      <c r="D157" s="93"/>
-      <c r="E157" s="93"/>
-      <c r="F157" s="93"/>
-      <c r="G157" s="93"/>
-      <c r="H157" s="93"/>
-      <c r="I157" s="93"/>
-      <c r="J157" s="72"/>
-      <c r="K157" s="78"/>
-      <c r="L157" s="78"/>
-      <c r="M157" s="78"/>
-      <c r="N157" s="78"/>
-      <c r="O157" s="78"/>
-      <c r="P157" s="78"/>
-      <c r="Q157" s="78"/>
-      <c r="R157" s="78"/>
-      <c r="S157" s="78"/>
-      <c r="T157" s="78"/>
-      <c r="U157" s="78"/>
-      <c r="V157" s="78"/>
-      <c r="W157" s="80"/>
-      <c r="X157" s="100"/>
-      <c r="Y157" s="100"/>
-      <c r="Z157" s="82"/>
-      <c r="AA157" s="100"/>
-      <c r="AB157" s="100"/>
-      <c r="AC157" s="101"/>
-      <c r="AD157" s="101"/>
-      <c r="AE157" s="101"/>
-      <c r="AF157" s="98"/>
+      <c r="A157" s="68" t="s">
+        <v>489</v>
+      </c>
+      <c r="B157" s="93">
+        <v>400</v>
+      </c>
+      <c r="C157" s="93" t="s">
+        <v>522</v>
+      </c>
+      <c r="D157" s="93">
+        <v>500</v>
+      </c>
+      <c r="E157" s="93">
+        <v>1750</v>
+      </c>
+      <c r="F157" s="93">
+        <v>2700</v>
+      </c>
+      <c r="G157" s="93" t="s">
+        <v>511</v>
+      </c>
+      <c r="H157" s="93" t="s">
+        <v>512</v>
+      </c>
+      <c r="I157" s="93">
+        <v>3000</v>
+      </c>
+      <c r="J157" s="72" t="s">
+        <v>512</v>
+      </c>
+      <c r="K157" s="78" t="s">
+        <v>513</v>
+      </c>
+      <c r="L157" s="78" t="s">
+        <v>514</v>
+      </c>
+      <c r="M157" s="78" t="s">
+        <v>515</v>
+      </c>
+      <c r="N157" s="78" t="s">
+        <v>516</v>
+      </c>
+      <c r="O157" s="78">
+        <v>0</v>
+      </c>
+      <c r="P157" s="78" t="s">
+        <v>517</v>
+      </c>
+      <c r="Q157" s="78" t="s">
+        <v>518</v>
+      </c>
+      <c r="R157" s="78" t="s">
+        <v>519</v>
+      </c>
+      <c r="S157" s="78" t="s">
+        <v>520</v>
+      </c>
+      <c r="T157" s="78" t="s">
+        <v>521</v>
+      </c>
+      <c r="U157" s="78">
+        <v>0</v>
+      </c>
+      <c r="V157" s="78" t="s">
+        <v>497</v>
+      </c>
+      <c r="W157" s="80">
+        <v>5000</v>
+      </c>
+      <c r="X157" s="100">
+        <v>6000</v>
+      </c>
+      <c r="Y157" s="100" t="s">
+        <v>498</v>
+      </c>
+      <c r="Z157" s="82">
+        <v>154</v>
+      </c>
+      <c r="AA157" s="100">
+        <v>240</v>
+      </c>
+      <c r="AB157" s="100">
+        <v>1</v>
+      </c>
+      <c r="AC157" s="101">
+        <v>400</v>
+      </c>
+      <c r="AD157" s="101">
+        <v>1</v>
+      </c>
+      <c r="AE157" s="101">
+        <v>93</v>
+      </c>
+      <c r="AF157" s="98" t="s">
+        <v>499</v>
+      </c>
+      <c r="AG157" s="44">
+        <v>1750</v>
+      </c>
+      <c r="AH157" s="44" t="s">
+        <v>500</v>
+      </c>
     </row>
     <row r="158" spans="1:36" s="44" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A158" s="68"/>
-      <c r="B158" s="93"/>
-      <c r="C158" s="93"/>
-      <c r="D158" s="93"/>
-      <c r="E158" s="93"/>
-      <c r="F158" s="93"/>
-      <c r="G158" s="93"/>
-      <c r="H158" s="93"/>
-      <c r="I158" s="93"/>
-      <c r="J158" s="72"/>
-      <c r="K158" s="78"/>
-      <c r="L158" s="78"/>
-      <c r="M158" s="78"/>
-      <c r="N158" s="78"/>
-      <c r="O158" s="78"/>
-      <c r="P158" s="78"/>
-      <c r="Q158" s="78"/>
-      <c r="R158" s="78"/>
-      <c r="S158" s="78"/>
-      <c r="T158" s="78"/>
-      <c r="U158" s="78"/>
-      <c r="V158" s="78"/>
-      <c r="W158" s="80"/>
-      <c r="X158" s="100"/>
-      <c r="Y158" s="100"/>
-      <c r="Z158" s="82"/>
-      <c r="AA158" s="100"/>
-      <c r="AB158" s="100"/>
-      <c r="AC158" s="101"/>
-      <c r="AD158" s="101"/>
-      <c r="AE158" s="101"/>
-      <c r="AF158" s="98"/>
+      <c r="A158" s="68" t="s">
+        <v>489</v>
+      </c>
+      <c r="B158" s="93">
+        <v>400</v>
+      </c>
+      <c r="C158" s="93" t="s">
+        <v>523</v>
+      </c>
+      <c r="D158" s="93">
+        <v>600</v>
+      </c>
+      <c r="E158" s="93">
+        <v>1800</v>
+      </c>
+      <c r="F158" s="93">
+        <v>2850</v>
+      </c>
+      <c r="G158" s="93" t="s">
+        <v>524</v>
+      </c>
+      <c r="H158" s="93" t="s">
+        <v>525</v>
+      </c>
+      <c r="I158" s="93">
+        <v>3200</v>
+      </c>
+      <c r="J158" s="72" t="s">
+        <v>525</v>
+      </c>
+      <c r="K158" s="78" t="s">
+        <v>526</v>
+      </c>
+      <c r="L158" s="78" t="s">
+        <v>527</v>
+      </c>
+      <c r="M158" s="78" t="s">
+        <v>528</v>
+      </c>
+      <c r="N158" s="78" t="s">
+        <v>529</v>
+      </c>
+      <c r="O158" s="78">
+        <v>0</v>
+      </c>
+      <c r="P158" s="78" t="s">
+        <v>530</v>
+      </c>
+      <c r="Q158" s="78" t="s">
+        <v>531</v>
+      </c>
+      <c r="R158" s="78" t="s">
+        <v>532</v>
+      </c>
+      <c r="S158" s="78" t="s">
+        <v>533</v>
+      </c>
+      <c r="T158" s="78" t="s">
+        <v>534</v>
+      </c>
+      <c r="U158" s="78">
+        <v>0</v>
+      </c>
+      <c r="V158" s="78" t="s">
+        <v>497</v>
+      </c>
+      <c r="W158" s="80">
+        <v>5000</v>
+      </c>
+      <c r="X158" s="100">
+        <v>6000</v>
+      </c>
+      <c r="Y158" s="100" t="s">
+        <v>498</v>
+      </c>
+      <c r="Z158" s="82">
+        <v>154</v>
+      </c>
+      <c r="AA158" s="100">
+        <v>240</v>
+      </c>
+      <c r="AB158" s="100">
+        <v>1</v>
+      </c>
+      <c r="AC158" s="101">
+        <v>400</v>
+      </c>
+      <c r="AD158" s="101">
+        <v>1</v>
+      </c>
+      <c r="AE158" s="101">
+        <v>117</v>
+      </c>
+      <c r="AF158" s="98" t="s">
+        <v>499</v>
+      </c>
+      <c r="AG158" s="44">
+        <v>1800</v>
+      </c>
+      <c r="AH158" s="44" t="s">
+        <v>500</v>
+      </c>
     </row>
     <row r="159" spans="1:36" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A159" s="32"/>
@@ -18253,6 +18668,7 @@
       <c r="N160" s="24"/>
       <c r="O160" s="24"/>
       <c r="P160" s="24"/>
+      <c r="Q160" s="24"/>
       <c r="R160" s="24"/>
       <c r="S160" s="24"/>
       <c r="T160" s="24"/>
@@ -18279,6 +18695,7 @@
       <c r="G161" s="27"/>
       <c r="H161" s="27"/>
       <c r="J161" s="24"/>
+      <c r="K161" s="24"/>
       <c r="L161" s="24"/>
       <c r="M161" s="24"/>
       <c r="N161" s="24"/>
@@ -18310,7 +18727,8 @@
       <c r="F162" s="27"/>
       <c r="G162" s="27"/>
       <c r="H162" s="27"/>
-      <c r="J162" s="24"/>
+      <c r="I162" s="24"/>
+      <c r="J162" s="27"/>
       <c r="K162" s="24"/>
       <c r="L162" s="24"/>
       <c r="M162" s="24"/>
@@ -18343,7 +18761,7 @@
       <c r="F163" s="27"/>
       <c r="G163" s="27"/>
       <c r="H163" s="27"/>
-      <c r="I163" s="24"/>
+      <c r="I163" s="27"/>
       <c r="J163" s="27"/>
       <c r="K163" s="24"/>
       <c r="L163" s="24"/>
@@ -18604,7 +19022,9 @@
       <c r="AC170" s="31"/>
       <c r="AD170" s="31"/>
       <c r="AE170" s="31"/>
-      <c r="AF170" s="36"/>
+      <c r="AF170" s="37"/>
+      <c r="AG170" s="45"/>
+      <c r="AH170" s="45"/>
     </row>
     <row r="171" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A171" s="32"/>
@@ -18638,9 +19058,7 @@
       <c r="AC171" s="31"/>
       <c r="AD171" s="31"/>
       <c r="AE171" s="31"/>
-      <c r="AF171" s="37"/>
-      <c r="AG171" s="45"/>
-      <c r="AH171" s="45"/>
+      <c r="AF171" s="36"/>
     </row>
     <row r="172" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A172" s="32"/>
@@ -18744,7 +19162,7 @@
       <c r="AE174" s="31"/>
       <c r="AF174" s="36"/>
     </row>
-    <row r="175" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:34" s="46" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A175" s="32"/>
       <c r="B175" s="27"/>
       <c r="C175" s="33"/>
@@ -18776,9 +19194,9 @@
       <c r="AC175" s="31"/>
       <c r="AD175" s="31"/>
       <c r="AE175" s="31"/>
-      <c r="AF175" s="36"/>
-    </row>
-    <row r="176" spans="1:34" s="46" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AF175" s="38"/>
+    </row>
+    <row r="176" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A176" s="32"/>
       <c r="B176" s="27"/>
       <c r="C176" s="33"/>
@@ -18811,8 +19229,10 @@
       <c r="AD176" s="31"/>
       <c r="AE176" s="31"/>
       <c r="AF176" s="38"/>
-    </row>
-    <row r="177" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AG176" s="46"/>
+      <c r="AH176" s="46"/>
+    </row>
+    <row r="177" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A177" s="32"/>
       <c r="B177" s="27"/>
       <c r="C177" s="33"/>
@@ -18844,11 +19264,9 @@
       <c r="AC177" s="31"/>
       <c r="AD177" s="31"/>
       <c r="AE177" s="31"/>
-      <c r="AF177" s="38"/>
-      <c r="AG177" s="46"/>
-      <c r="AH177" s="46"/>
-    </row>
-    <row r="178" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AF177" s="36"/>
+    </row>
+    <row r="178" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A178" s="32"/>
       <c r="B178" s="27"/>
       <c r="C178" s="33"/>
@@ -18882,41 +19300,42 @@
       <c r="AE178" s="31"/>
       <c r="AF178" s="36"/>
     </row>
-    <row r="179" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A179" s="32"/>
-      <c r="B179" s="27"/>
-      <c r="C179" s="33"/>
-      <c r="D179" s="27"/>
-      <c r="E179" s="27"/>
-      <c r="F179" s="27"/>
-      <c r="G179" s="27"/>
-      <c r="H179" s="27"/>
-      <c r="I179" s="27"/>
-      <c r="J179" s="27"/>
-      <c r="K179" s="24"/>
-      <c r="L179" s="24"/>
-      <c r="M179" s="24"/>
-      <c r="N179" s="24"/>
-      <c r="O179" s="24"/>
-      <c r="P179" s="24"/>
-      <c r="Q179" s="24"/>
-      <c r="R179" s="24"/>
-      <c r="S179" s="24"/>
-      <c r="T179" s="24"/>
-      <c r="U179" s="24"/>
-      <c r="V179" s="24"/>
-      <c r="W179" s="29"/>
-      <c r="X179" s="30"/>
-      <c r="Y179" s="30"/>
-      <c r="Z179" s="26"/>
-      <c r="AA179" s="30"/>
-      <c r="AB179" s="30"/>
-      <c r="AC179" s="31"/>
-      <c r="AD179" s="31"/>
-      <c r="AE179" s="31"/>
-      <c r="AF179" s="36"/>
-    </row>
-    <row r="180" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A179" s="35"/>
+      <c r="B179" s="23"/>
+      <c r="C179" s="40"/>
+      <c r="D179" s="40"/>
+      <c r="E179" s="41"/>
+      <c r="F179" s="41"/>
+      <c r="G179" s="41"/>
+      <c r="H179" s="42"/>
+      <c r="I179" s="42"/>
+      <c r="J179" s="42"/>
+      <c r="K179" s="43"/>
+      <c r="L179" s="43"/>
+      <c r="M179" s="43"/>
+      <c r="N179" s="43"/>
+      <c r="O179" s="43"/>
+      <c r="P179" s="43"/>
+      <c r="Q179" s="43"/>
+      <c r="R179" s="43"/>
+      <c r="S179" s="43"/>
+      <c r="T179" s="43"/>
+      <c r="U179" s="43"/>
+      <c r="V179" s="43"/>
+      <c r="W179" s="42"/>
+      <c r="X179" s="42"/>
+      <c r="Y179" s="42"/>
+      <c r="Z179" s="42"/>
+      <c r="AA179" s="42"/>
+      <c r="AB179" s="42"/>
+      <c r="AC179" s="36"/>
+      <c r="AD179" s="36"/>
+      <c r="AE179" s="36"/>
+      <c r="AF179" s="42"/>
+      <c r="AG179" s="36"/>
+    </row>
+    <row r="180" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A180" s="35"/>
       <c r="B180" s="23"/>
       <c r="C180" s="40"/>
@@ -18951,7 +19370,7 @@
       <c r="AF180" s="42"/>
       <c r="AG180" s="36"/>
     </row>
-    <row r="181" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A181" s="35"/>
       <c r="B181" s="23"/>
       <c r="C181" s="40"/>
@@ -18986,7 +19405,7 @@
       <c r="AF181" s="42"/>
       <c r="AG181" s="36"/>
     </row>
-    <row r="182" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A182" s="35"/>
       <c r="B182" s="23"/>
       <c r="C182" s="40"/>
@@ -19021,7 +19440,7 @@
       <c r="AF182" s="42"/>
       <c r="AG182" s="36"/>
     </row>
-    <row r="183" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A183" s="35"/>
       <c r="B183" s="23"/>
       <c r="C183" s="40"/>
@@ -19056,7 +19475,7 @@
       <c r="AF183" s="42"/>
       <c r="AG183" s="36"/>
     </row>
-    <row r="184" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A184" s="35"/>
       <c r="B184" s="23"/>
       <c r="C184" s="40"/>
@@ -19091,7 +19510,7 @@
       <c r="AF184" s="42"/>
       <c r="AG184" s="36"/>
     </row>
-    <row r="185" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A185" s="35"/>
       <c r="B185" s="23"/>
       <c r="C185" s="40"/>
@@ -19126,7 +19545,7 @@
       <c r="AF185" s="42"/>
       <c r="AG185" s="36"/>
     </row>
-    <row r="186" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A186" s="35"/>
       <c r="B186" s="23"/>
       <c r="C186" s="40"/>
@@ -19161,7 +19580,7 @@
       <c r="AF186" s="42"/>
       <c r="AG186" s="36"/>
     </row>
-    <row r="187" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A187" s="35"/>
       <c r="B187" s="23"/>
       <c r="C187" s="40"/>
@@ -19196,7 +19615,7 @@
       <c r="AF187" s="42"/>
       <c r="AG187" s="36"/>
     </row>
-    <row r="188" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A188" s="35"/>
       <c r="B188" s="23"/>
       <c r="C188" s="40"/>
@@ -19231,7 +19650,7 @@
       <c r="AF188" s="42"/>
       <c r="AG188" s="36"/>
     </row>
-    <row r="189" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A189" s="35"/>
       <c r="B189" s="23"/>
       <c r="C189" s="40"/>
@@ -19266,7 +19685,7 @@
       <c r="AF189" s="42"/>
       <c r="AG189" s="36"/>
     </row>
-    <row r="190" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A190" s="35"/>
       <c r="B190" s="23"/>
       <c r="C190" s="40"/>
@@ -19301,7 +19720,7 @@
       <c r="AF190" s="42"/>
       <c r="AG190" s="36"/>
     </row>
-    <row r="191" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A191" s="35"/>
       <c r="B191" s="23"/>
       <c r="C191" s="40"/>
@@ -19336,7 +19755,7 @@
       <c r="AF191" s="42"/>
       <c r="AG191" s="36"/>
     </row>
-    <row r="192" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A192" s="35"/>
       <c r="B192" s="23"/>
       <c r="C192" s="40"/>
@@ -19792,7 +20211,7 @@
       <c r="AG204" s="36"/>
     </row>
     <row r="205" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A205" s="35"/>
+      <c r="A205" s="39"/>
       <c r="B205" s="23"/>
       <c r="C205" s="40"/>
       <c r="D205" s="40"/>
@@ -24202,7 +24621,6 @@
       <c r="AG330" s="36"/>
     </row>
     <row r="331" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A331" s="39"/>
       <c r="B331" s="23"/>
       <c r="C331" s="40"/>
       <c r="D331" s="40"/>
@@ -49974,7 +50392,7 @@
       <c r="AF1088" s="42"/>
       <c r="AG1088" s="36"/>
     </row>
-    <row r="1089" spans="2:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1089" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B1089" s="23"/>
       <c r="C1089" s="40"/>
       <c r="D1089" s="40"/>
@@ -50008,7 +50426,7 @@
       <c r="AF1089" s="42"/>
       <c r="AG1089" s="36"/>
     </row>
-    <row r="1090" spans="2:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1090" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B1090" s="23"/>
       <c r="C1090" s="40"/>
       <c r="D1090" s="40"/>
@@ -50042,7 +50460,7 @@
       <c r="AF1090" s="42"/>
       <c r="AG1090" s="36"/>
     </row>
-    <row r="1091" spans="2:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1091" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B1091" s="23"/>
       <c r="C1091" s="40"/>
       <c r="D1091" s="40"/>
@@ -50076,7 +50494,7 @@
       <c r="AF1091" s="42"/>
       <c r="AG1091" s="36"/>
     </row>
-    <row r="1092" spans="2:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1092" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B1092" s="23"/>
       <c r="C1092" s="40"/>
       <c r="D1092" s="40"/>
@@ -50110,7 +50528,7 @@
       <c r="AF1092" s="42"/>
       <c r="AG1092" s="36"/>
     </row>
-    <row r="1093" spans="2:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1093" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B1093" s="23"/>
       <c r="C1093" s="40"/>
       <c r="D1093" s="40"/>
@@ -50144,7 +50562,7 @@
       <c r="AF1093" s="42"/>
       <c r="AG1093" s="36"/>
     </row>
-    <row r="1094" spans="2:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1094" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B1094" s="23"/>
       <c r="C1094" s="40"/>
       <c r="D1094" s="40"/>
@@ -50178,7 +50596,7 @@
       <c r="AF1094" s="42"/>
       <c r="AG1094" s="36"/>
     </row>
-    <row r="1095" spans="2:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1095" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B1095" s="23"/>
       <c r="C1095" s="40"/>
       <c r="D1095" s="40"/>
@@ -50212,7 +50630,7 @@
       <c r="AF1095" s="42"/>
       <c r="AG1095" s="36"/>
     </row>
-    <row r="1096" spans="2:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1096" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B1096" s="23"/>
       <c r="C1096" s="40"/>
       <c r="D1096" s="40"/>
@@ -50246,7 +50664,7 @@
       <c r="AF1096" s="42"/>
       <c r="AG1096" s="36"/>
     </row>
-    <row r="1097" spans="2:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1097" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B1097" s="23"/>
       <c r="C1097" s="40"/>
       <c r="D1097" s="40"/>
@@ -50280,7 +50698,7 @@
       <c r="AF1097" s="42"/>
       <c r="AG1097" s="36"/>
     </row>
-    <row r="1098" spans="2:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1098" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B1098" s="23"/>
       <c r="C1098" s="40"/>
       <c r="D1098" s="40"/>
@@ -50314,7 +50732,7 @@
       <c r="AF1098" s="42"/>
       <c r="AG1098" s="36"/>
     </row>
-    <row r="1099" spans="2:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1099" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B1099" s="23"/>
       <c r="C1099" s="40"/>
       <c r="D1099" s="40"/>
@@ -50348,7 +50766,7 @@
       <c r="AF1099" s="42"/>
       <c r="AG1099" s="36"/>
     </row>
-    <row r="1100" spans="2:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1100" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B1100" s="23"/>
       <c r="C1100" s="40"/>
       <c r="D1100" s="40"/>
@@ -50382,7 +50800,7 @@
       <c r="AF1100" s="42"/>
       <c r="AG1100" s="36"/>
     </row>
-    <row r="1101" spans="2:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1101" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B1101" s="23"/>
       <c r="C1101" s="40"/>
       <c r="D1101" s="40"/>
@@ -50416,7 +50834,7 @@
       <c r="AF1101" s="42"/>
       <c r="AG1101" s="36"/>
     </row>
-    <row r="1102" spans="2:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1102" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B1102" s="23"/>
       <c r="C1102" s="40"/>
       <c r="D1102" s="40"/>
@@ -50450,7 +50868,7 @@
       <c r="AF1102" s="42"/>
       <c r="AG1102" s="36"/>
     </row>
-    <row r="1103" spans="2:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1103" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B1103" s="23"/>
       <c r="C1103" s="40"/>
       <c r="D1103" s="40"/>
@@ -50484,8 +50902,9 @@
       <c r="AF1103" s="42"/>
       <c r="AG1103" s="36"/>
     </row>
-    <row r="1104" spans="2:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B1104" s="23"/>
+    <row r="1104" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1104" s="34"/>
+      <c r="B1104" s="40"/>
       <c r="C1104" s="40"/>
       <c r="D1104" s="40"/>
       <c r="E1104" s="41"/>
@@ -50518,53 +50937,18 @@
       <c r="AF1104" s="42"/>
       <c r="AG1104" s="36"/>
     </row>
-    <row r="1105" spans="1:33" s="44" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1105" s="34"/>
-      <c r="B1105" s="40"/>
-      <c r="C1105" s="40"/>
-      <c r="D1105" s="40"/>
-      <c r="E1105" s="41"/>
-      <c r="F1105" s="41"/>
-      <c r="G1105" s="41"/>
-      <c r="H1105" s="42"/>
-      <c r="I1105" s="42"/>
-      <c r="J1105" s="42"/>
-      <c r="K1105" s="43"/>
-      <c r="L1105" s="43"/>
-      <c r="M1105" s="43"/>
-      <c r="N1105" s="43"/>
-      <c r="O1105" s="43"/>
-      <c r="P1105" s="43"/>
-      <c r="Q1105" s="43"/>
-      <c r="R1105" s="43"/>
-      <c r="S1105" s="43"/>
-      <c r="T1105" s="43"/>
-      <c r="U1105" s="43"/>
-      <c r="V1105" s="43"/>
-      <c r="W1105" s="42"/>
-      <c r="X1105" s="42"/>
-      <c r="Y1105" s="42"/>
-      <c r="Z1105" s="42"/>
-      <c r="AA1105" s="42"/>
-      <c r="AB1105" s="42"/>
-      <c r="AC1105" s="36"/>
-      <c r="AD1105" s="36"/>
-      <c r="AE1105" s="36"/>
-      <c r="AF1105" s="42"/>
-      <c r="AG1105" s="36"/>
-    </row>
   </sheetData>
   <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter 1 for gas handler" sqref="AH5:AH117" xr:uid="{D4F63CA9-4B8A-4E8D-8A06-46E288212DB9}">
-      <formula1>$A$1001:$A$1002</formula1>
+      <formula1>$A$1000:$A$1001</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter 1 for obsolete" sqref="AG5:AG117 AG180:AG1104 AF118:AF149 AF152:AF179" xr:uid="{6AE47EA0-4762-42E9-B62C-07E716141A03}">
-      <formula1>$A$1001:$A$1002</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter 1 for obsolete" sqref="AG5:AG117 AF152:AF178 AF118:AF149 AG179:AG1103" xr:uid="{6AE47EA0-4762-42E9-B62C-07E716141A03}">
+      <formula1>$A$1000:$A$1001</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Important Notice:" prompt="If a manufacturer is not the SubPUMP databank, this field is required. The available manufacturers within SubPUMP can be found in the drop down list in the manufacturer field (Column B)." sqref="W39 W82:W97 W7:W34 W42:W77 W79:W80 W99:W100 W103:W117" xr:uid="{3ABA8888-4F6D-4392-92AF-AB8BE0A86DDD}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Important Notice:" prompt="-------_x000a_If a manufacturer is not in SubPUMP databank, this field is required._x000a_-------_x000a_Manufacturers in SubPUMP:_x000a_Almaz, Alnas, Borets, CAI, Centrilift/ODI or CLift, ESP, Lemaz, Novomet, Novo, ODI, Schlumberger/Reda or Reda, Weatherford or Wford, WSP" sqref="W180:W1104 V176:V179 V118:V149 V162:V174 V152:V160" xr:uid="{9A547A56-E420-4C2C-BE7C-866904004891}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Manufacturer Name" prompt="Select a manufacturer from the list, or enter a new manufacturer using a short name" sqref="B180:B1104 A152:A179" xr:uid="{730E29A7-E193-4760-8A9E-D7881A70E46B}">
-      <formula1>$A$1010:$A$1022</formula1>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Important Notice:" prompt="-------_x000a_If a manufacturer is not in SubPUMP databank, this field is required._x000a_-------_x000a_Manufacturers in SubPUMP:_x000a_Almaz, Alnas, Borets, CAI, Centrilift/ODI or CLift, ESP, Lemaz, Novomet, Novo, ODI, Schlumberger/Reda or Reda, Weatherford or Wford, WSP" sqref="W179:W1103 V175:V178 V118:V149 V161:V173 V152:V159" xr:uid="{9A547A56-E420-4C2C-BE7C-866904004891}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Manufacturer Name" prompt="Select a manufacturer from the list, or enter a new manufacturer using a short name" sqref="B179:B1103 A152:A178" xr:uid="{730E29A7-E193-4760-8A9E-D7881A70E46B}">
+      <formula1>$A$1009:$A$1021</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>